<commit_message>
fix ai and review exam
</commit_message>
<xml_diff>
--- a/uploads/reports/monthly_report_2026-02.xlsx
+++ b/uploads/reports/monthly_report_2026-02.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="184">
   <si>
     <t>AttemptId</t>
   </si>
@@ -47,22 +47,132 @@
     <t>AiFeedback</t>
   </si>
   <si>
+    <t>87</t>
+  </si>
+  <si>
+    <t>91</t>
+  </si>
+  <si>
+    <t>hoanganhnd2003@gmail.com</t>
+  </si>
+  <si>
+    <t>Hoàng Anh Nguyễn</t>
+  </si>
+  <si>
+    <t>94</t>
+  </si>
+  <si>
+    <t>PRACTICE</t>
+  </si>
+  <si>
+    <t>2026-02-04T16:51:08.886226</t>
+  </si>
+  <si>
+    <t>2026-02-04T16:52:06.301896</t>
+  </si>
+  <si>
+    <t>[{"questionId":829,"questionType":"ESSAY","selectedAnswer":null,"correctAnswer":null,"textAnswer":"sadsa","sampleAnswer":"Tài liệu chỉ ra rằng Next.js có sự phân biệt giữa cơ chế server side và client side. Điều này ngụ ý rằng Next.js có thể xử lý việc render và tương tác ở cả phía máy chủ và phía trình duyệt. Khả năng này cho phép các chiến lược khác nhau trong việc xây dựng ứng dụng web, tận dụng ưu điểm của cả hai môi trường.","score":0,"maxScore":10,"feedback":"Chưa đúng ý trọng tâm."},{"questionId":830,"questionType":"MCQ","selectedAnswer":"C","correctAnswer":"C","textAnswer":null,"sampleAnswer":null,"score":10,"maxScore":10,"feedback":"Đúng"},{"questionId":831,"questionType":"MCQ","selectedAnswer":"B","correctAnswer":"B","textAnswer":null,"sampleAnswer":null,"score":10,"maxScore":10,"feedback":"Đúng"},{"questionId":832,"questionType":"ESSAY","selectedAnswer":null,"correctAnswer":null,"textAnswer":"sadsd","sampleAnswer":"Tài liệu liệt kê ba chức năng chính của `router dom`. Thứ nhất là \"router basic\", dùng cho định tuyến cơ bản. Thứ hai là \"router lấy tham số trên url\", cho phép trích xuất dữ liệu từ URL. Cuối cùng là \"chuyển hướng\", giúp điều hướng người dùng đến các trang khác trong ứng dụng.","score":0,"maxScore":10,"feedback":"Chưa đúng ý trọng tâm."},{"questionId":833,"questionType":"MCQ","selectedAnswer":"C","correctAnswer":"C","textAnswer":null,"sampleAnswer":null,"score":10,"maxScore":10,"feedback":"Đúng"},{"questionId":834,"questionType":"MCQ","selectedAnswer":"C","correctAnswer":"C","textAnswer":null,"sampleAnswer":null,"score":10,"maxScore":10,"feedback":"Đúng"},{"questionId":835,"questionType":"ESSAY","selectedAnswer":null,"correctAnswer":null,"textAnswer":"sadsada","sampleAnswer":"Theo tài liệu, Redux bao gồm các thành phần cơ bản và đặc biệt là thư viện Redux Toolkit. Redux Toolkit được giới thiệu như một bộ công cụ giúp đơn giản hóa quá trình phát triển Redux. Nó cung cấp các tiện ích để viết code Redux hiệu quả và dễ dàng hơn, giúp giảm bớt boilerplate code.","score":0,"maxScore":10,"feedback":"Chưa đúng ý trọng tâm."},{"questionId":836,"questionType":"MCQ","selectedAnswer":"C","correctAnswer":"C","textAnswer":null,"sampleAnswer":null,"score":10,"maxScore":10,"feedback":"Đúng"},{"questionId":837,"questionType":"MCQ","selectedAnswer":"B","correctAnswer":"B","textAnswer":null,"sampleAnswer":null,"score":10,"maxScore":10,"feedback":"Đúng"},{"questionId":838,"questionType":"MCQ","selectedAnswer":"C","correctAnswer":"B","textAnswer":null,"sampleAnswer":null,"score":0,"maxScore":10,"feedback":"Sai"}]</t>
+  </si>
+  <si>
+    <t>Chào Hoàng Anh Nguyễn,
+- Chào Hoàng Anh Nguyễn.
+- Điểm tổng: 60/100
+- Điểm tổng 60/100 cho thấy bạn có nắm được một phần kiến thức cơ bản.
+- Bạn làm khá tốt các câu hỏi trắc nghiệm nhưng còn gặp nhiều khó khăn ở các câu hỏi tự luận.
+- Lỗi sai nổi bật nhất là bạn đã bỏ trống hoặc điền câu trả lời không liên quan cho tất cả các câu hỏi tự luận (Câu 1, 4, 7).
+- Điều này cho thấy bạn chưa nắm vững kiến thức chuyên sâu hoặc kỹ năng trình bày các khái niệm được yêu cầu giải thích.
+- Bạn còn sai một câu hỏi trắc nghiệm về `router dom` (Câu 10).
+- Hãy tập trung ôn luyện lại các khái niệm yêu cầu giải thích chi tiết, đặc biệt là về Next.js (phân biệt server/client side) và các chức năng của `router dom`.</t>
+  </si>
+  <si>
+    <t>86</t>
+  </si>
+  <si>
+    <t>93</t>
+  </si>
+  <si>
+    <t>2026-02-04T16:48:23.802722</t>
+  </si>
+  <si>
+    <t>2026-02-04T16:49:42.780638</t>
+  </si>
+  <si>
+    <t>[{"questionId":819,"questionType":"MCQ","selectedAnswer":"B","correctAnswer":"B","textAnswer":null,"sampleAnswer":null,"score":10,"maxScore":10,"feedback":"Đúng"},{"questionId":820,"questionType":"ESSAY","selectedAnswer":null,"correctAnswer":null,"textAnswer":"ádasf","sampleAnswer":"Tài liệu chỉ ra rằng Next.js có sự phân biệt giữa cơ chế server side và client side. Điều này ngụ ý rằng Next.js có thể xử lý việc render và tương tác ở cả phía máy chủ và phía trình duyệt, cho phép các chiến lược khác nhau trong việc xây dựng ứng dụng web.","score":0,"maxScore":10,"feedback":"Chưa đúng ý trọng tâm."},{"questionId":821,"questionType":"MCQ","selectedAnswer":"C","correctAnswer":"C","textAnswer":null,"sampleAnswer":null,"score":10,"maxScore":10,"feedback":"Đúng"},{"questionId":822,"questionType":"MCQ","selectedAnswer":"C","correctAnswer":"C","textAnswer":null,"sampleAnswer":null,"score":10,"maxScore":10,"feedback":"Đúng"},{"questionId":823,"questionType":"ESSAY","selectedAnswer":null,"correctAnswer":null,"textAnswer":"sad","sampleAnswer":"Theo tài liệu, Redux bao gồm các thành phần cơ bản và đặc biệt là thư viện Redux Toolkit. Redux Toolkit được giới thiệu như một bộ công cụ giúp đơn giản hóa quá trình phát triển Redux, cung cấp các tiện ích để viết code Redux hiệu quả hơn.","score":0,"maxScore":10,"feedback":"Chưa đúng ý trọng tâm."},{"questionId":824,"questionType":"MCQ","selectedAnswer":"D","correctAnswer":"D","textAnswer":null,"sampleAnswer":null,"score":10,"maxScore":10,"feedback":"Đúng"},{"questionId":825,"questionType":"MCQ","selectedAnswer":"B","correctAnswer":"C","textAnswer":null,"sampleAnswer":null,"score":0,"maxScore":10,"feedback":"Sai"},{"questionId":826,"questionType":"ESSAY","selectedAnswer":null,"correctAnswer":null,"textAnswer":"ádsad","sampleAnswer":"Tài liệu liệt kê ba chức năng chính của `router dom`. Đó là 'router basic' (định tuyến cơ bản), 'router lấy tham số trên url' (khả năng trích xuất dữ liệu từ URL), và 'chuyển hướng' (khả năng điều hướng người dùng đến các trang khác).","score":0,"maxScore":10,"feedback":"Chưa đúng ý trọng tâm."},{"questionId":827,"questionType":"MCQ","selectedAnswer":"B","correctAnswer":"B","textAnswer":null,"sampleAnswer":null,"score":10,"maxScore":10,"feedback":"Đúng"},{"questionId":828,"questionType":"MCQ","selectedAnswer":"C","correctAnswer":"C","textAnswer":null,"sampleAnswer":null,"score":10,"maxScore":10,"feedback":"Đúng"}]</t>
+  </si>
+  <si>
+    <t>Chào Hoàng Anh Nguyễn,
+- Chào Hoàng Anh Nguyễn.
+- Điểm tổng: 60/100
+- Bạn đã đạt được điểm khá ở phần trắc nghiệm, cho thấy bạn có nắm vững một số kiến thức cơ bản trong tài liệu.
+- Tuy nhiên, bạn cần cải thiện đáng kể ở các câu hỏi tự luận và diễn giải.
+- Lỗi sai nổi bật nhất là khả năng trả lời các câu hỏi tự luận, khi tất cả các câu hỏi dạng này đều chưa được trả lời đúng hoặc đầy đủ.
+- Bạn gặp khó khăn trong việc tổng hợp và diễn đạt thông tin từ tài liệu cho các khái niệm như cơ chế server/client side trong Next.js hay các thành phần của Redux.
+- Có một câu hỏi trắc nghiệm về phân biệt cơ chế trong Next.js bạn chọn sai, cho thấy cần xem xét kỹ hơn về chủ đề này.
+- Hãy dành thời gian đọc kỹ và sâu hơn các tài liệu, đặc biệt là các phần giải thích khái niệm và cơ chế.</t>
+  </si>
+  <si>
+    <t>85</t>
+  </si>
+  <si>
+    <t>92</t>
+  </si>
+  <si>
+    <t>2026-02-04T14:36:12.424293</t>
+  </si>
+  <si>
+    <t>2026-02-04T14:36:54.229126</t>
+  </si>
+  <si>
+    <t>[{"questionId":809,"questionType":"MCQ","selectedAnswer":"C","correctAnswer":"B","textAnswer":null,"sampleAnswer":null,"score":0,"maxScore":10,"feedback":"Sai"},{"questionId":810,"questionType":"ESSAY","selectedAnswer":null,"correctAnswer":null,"textAnswer":"sadasd","sampleAnswer":"IoC Container là thành phần lõi của Spring, chịu trách nhiệm tạo bean, inject dependency và quản lý vòng đời bean. Nó đảm bảo các object được khởi tạo và liên kết đúng cách. Hai loại IoC Container phổ biến là BeanFactory (cơ bản, nhẹ) và ApplicationContext (nâng cao, dùng phổ biến, mặc định trong Spring Boot).","score":0,"maxScore":10,"feedback":"Chưa đúng ý trọng tâm."},{"questionId":811,"questionType":"MCQ","selectedAnswer":"B","correctAnswer":"B","textAnswer":null,"sampleAnswer":null,"score":10,"maxScore":10,"feedback":"Đúng"},{"questionId":812,"questionType":"MCQ","selectedAnswer":"C","correctAnswer":"C","textAnswer":null,"sampleAnswer":null,"score":10,"maxScore":10,"feedback":"Đúng"},{"questionId":813,"questionType":"ESSAY","selectedAnswer":null,"correctAnswer":null,"textAnswer":"dfasf","sampleAnswer":"Client gửi request cho DispatcherServlet. DispatcherServlet sử dụng HandlerMapping để ánh xạ tới Controller phù hợp. Controller gọi các phương thức xử lý, thiết lập Model dữ liệu và trả về tên View. DispatcherServlet dùng ViewResolver để xác định View, sau đó chuyển Model cho View để render và trả HTTP response về cho Client.","score":0,"maxScore":10,"feedback":"Chưa đúng ý trọng tâm."},{"questionId":814,"questionType":"MCQ","selectedAnswer":"B","correctAnswer":"B","textAnswer":null,"sampleAnswer":null,"score":10,"maxScore":10,"feedback":"Đúng"},{"questionId":815,"questionType":"MCQ","selectedAnswer":"C","correctAnswer":"C","textAnswer":null,"sampleAnswer":null,"score":10,"maxScore":10,"feedback":"Đúng"},{"questionId":816,"questionType":"ESSAY","selectedAnswer":null,"correctAnswer":null,"textAnswer":"sấd","sampleAnswer":"IoC là nguyên lý thiết kế trong đó Spring Framework chịu trách nhiệm tạo, quản lý, liên kết và huỷ object thay cho lập trình viên. Mục đích chính là đảo ngược quyền kiểm soát việc tạo dependency cho Spring. Các lợi ích bao gồm tránh phụ thuộc chặt giữa các class, dễ thay đổi implementation, dễ test (mock), và giúp code linh hoạt, dễ bảo trì.","score":0,"maxScore":10,"feedback":"Chưa đúng ý trọng tâm."},{"questionId":817,"questionType":"MCQ","selectedAnswer":"D","correctAnswer":"D","textAnswer":null,"sampleAnswer":null,"score":10,"maxScore":10,"feedback":"Đúng"},{"questionId":818,"questionType":"MCQ","selectedAnswer":"B","correctAnswer":"B","textAnswer":null,"sampleAnswer":null,"score":10,"maxScore":10,"feedback":"Đúng"}]</t>
+  </si>
+  <si>
+    <t>Chào Hoàng Anh Nguyễn,
+- Chào Hoàng Anh Nguyễn.
+- Điểm tổng 60/100 cho thấy bạn có nắm vững một số kiến thức cơ bản về Spring Framework.
+- Bạn làm tốt ở các câu hỏi trắc nghiệm về định nghĩa, annotation và vai trò của các thành phần riêng lẻ.
+- Tuy nhiên, bạn cần cải thiện đáng kể ở các câu hỏi tự luận và các nguyên lý cốt lõi của Spring.
+- Lỗi sai nổi bật:
+- Bạn chưa nắm vững nguyên lý Inversion of Control (IoC), mục đích và lợi ích của nó.
+- Kiến thức về vai trò chính và các loại IoC Container còn hạn chế.
+- Bạn gặp khó khăn trong việc mô tả luồng xử lý HTTP request trong Spring MVC.</t>
+  </si>
+  <si>
+    <t>84</t>
+  </si>
+  <si>
+    <t>103</t>
+  </si>
+  <si>
+    <t>hoanganhyb2003@gmail.com</t>
+  </si>
+  <si>
+    <t>Hoang Anh Nguyen</t>
+  </si>
+  <si>
+    <t>2026-02-04T14:19:22.551509</t>
+  </si>
+  <si>
+    <t>2026-02-04T14:24:42.867705</t>
+  </si>
+  <si>
+    <t>[{"questionId":799,"questionType":"MCQ","selectedAnswer":"C","correctAnswer":"C","textAnswer":null,"sampleAnswer":null,"score":10,"maxScore":10,"feedback":"Đúng"},{"questionId":800,"questionType":"ESSAY","selectedAnswer":null,"correctAnswer":null,"textAnswer":"server-side tạo HTML trên máy chủ, tối ưu SEO tốc độ tải đầu\nclient-side render bằng JavaScript bằng trình duyệt","sampleAnswer":"Trong Next.js, cơ chế server-side liên quan đến việc render trang trên máy chủ trước khi gửi đến trình duyệt, giúp cải thiện SEO và hiệu suất tải trang ban đầu. Ngược lại, cơ chế client-side là khi trang được render hoàn toàn trên trình duyệt của người dùng sau khi tải về, thường được sử dụng cho các tương tác động.","score":8,"maxScore":10,"feedback":"Thiếu ý: Next.js"},{"questionId":801,"questionType":"MCQ","selectedAnswer":"B","correctAnswer":"B","textAnswer":null,"sampleAnswer":null,"score":10,"maxScore":10,"feedback":"Đúng"},{"questionId":802,"questionType":"MCQ","selectedAnswer":"B","correctAnswer":"B","textAnswer":null,"sampleAnswer":null,"score":10,"maxScore":10,"feedback":"Đúng"},{"questionId":803,"questionType":"ESSAY","selectedAnswer":null,"correctAnswer":null,"textAnswer":"Redux là thư viện quản lý trạng \ncác thành phần chính là \nstore, action, reducer, reduxtoolkit","sampleAnswer":"Redux là một thư viện quản lý trạng thái ứng dụng. Các thành phần chính của Redux bao gồm store (nơi lưu trữ trạng thái), actions (các đối tượng mô tả sự kiện đã xảy ra), và reducers (các hàm thuần túy xác định cách trạng thái thay đổi để phản ứng với actions). Ngoài ra, tài liệu còn nhắc đến thư viện Redux Toolkit giúp đơn giản hóa việc sử dụng Redux.","score":4,"maxScore":10,"feedback":"Thiếu ý: actions, reducers, Redux Toolkit"},{"questionId":804,"questionType":"MCQ","selectedAnswer":"B","correctAnswer":"B","textAnswer":null,"sampleAnswer":null,"score":10,"maxScore":10,"feedback":"Đúng"},{"questionId":805,"questionType":"MCQ","selectedAnswer":"B","correctAnswer":"B","textAnswer":null,"sampleAnswer":null,"score":10,"maxScore":10,"feedback":"Đúng"},{"questionId":806,"questionType":"ESSAY","selectedAnswer":null,"correctAnswer":null,"textAnswer":"không biết","sampleAnswer":"Các chức năng cơ bản của router được đề cập bao gồm định tuyến cơ bản (router basic), khả năng lấy tham số từ URL (router lấy tham số trên url), và chức năng chuyển hướng (chuyển hướng).","score":0,"maxScore":10,"feedback":"Chưa đúng ý trọng tâm."},{"questionId":807,"questionType":"MCQ","selectedAnswer":"C","correctAnswer":"C","textAnswer":null,"sampleAnswer":null,"score":10,"maxScore":10,"feedback":"Đúng"},{"questionId":808,"questionType":"MCQ","selectedAnswer":"B","correctAnswer":"B","textAnswer":null,"sampleAnswer":null,"score":10,"maxScore":10,"feedback":"Đúng"}]</t>
+  </si>
+  <si>
+    <t>Chào Hoang Anh Nguyen,
+- Chào Hoang Anh Nguyen.
+- Điểm tổng: 82/100
+- Bạn có kết quả bài làm tốt với 82/100 điểm, cho thấy sự nắm vững kiến thức nền tảng.
+- Các câu hỏi trắc nghiệm đều được trả lời đúng, thể hiện khả năng ghi nhớ và nhận diện thông tin tốt.
+- Bạn cần chú ý cải thiện ở các câu hỏi tự luận để đạt điểm tối đa.
+- Phần giải thích về Redux (câu 5) chỉ liệt kê các thành phần mà chưa đi vào giải thích chi tiết vai trò của từng mục.
+- Bạn chưa nắm được hoặc bỏ trống câu hỏi về các chức năng cơ bản của router (câu 8).
+- Câu trả lời về server-side và client-side trong Next.js (câu 2) còn khá ngắn gọn, có thể bổ sung thêm chi tiết.</t>
+  </si>
+  <si>
     <t>83</t>
   </si>
   <si>
-    <t>91</t>
-  </si>
-  <si>
-    <t>hoanganhnd2003@gmail.com</t>
-  </si>
-  <si>
-    <t>Hoàng Anh Nguyễn</t>
-  </si>
-  <si>
     <t>90</t>
-  </si>
-  <si>
-    <t>PRACTICE</t>
   </si>
   <si>
     <t>2026-02-03T14:07:05.349100</t>
@@ -140,9 +250,6 @@
     <t>80</t>
   </si>
   <si>
-    <t>87</t>
-  </si>
-  <si>
     <t>2026-02-03T12:17:09.142761</t>
   </si>
   <si>
@@ -166,9 +273,6 @@
     <t>79</t>
   </si>
   <si>
-    <t>86</t>
-  </si>
-  <si>
     <t>2026-02-03T11:20:45.167648</t>
   </si>
   <si>
@@ -192,9 +296,6 @@
     <t>78</t>
   </si>
   <si>
-    <t>85</t>
-  </si>
-  <si>
     <t>2026-02-03T10:52:21.445947</t>
   </si>
   <si>
@@ -216,9 +317,6 @@
   </si>
   <si>
     <t>77</t>
-  </si>
-  <si>
-    <t>84</t>
   </si>
   <si>
     <t>2026-02-03T10:50:38.476897</t>
@@ -426,15 +524,6 @@
   </si>
   <si>
     <t>68</t>
-  </si>
-  <si>
-    <t>103</t>
-  </si>
-  <si>
-    <t>hoanganhyb2003@gmail.com</t>
-  </si>
-  <si>
-    <t>Hoang Anh Nguyen</t>
   </si>
   <si>
     <t>2026-02-02T14:04:37.691325</t>
@@ -770,7 +859,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="9.18359375" customWidth="true" bestFit="true"/>
@@ -847,7 +936,7 @@
         <v>18</v>
       </c>
       <c r="I2" t="n" s="0">
-        <v>40.0</v>
+        <v>60.0</v>
       </c>
       <c r="J2" t="s" s="0">
         <v>19</v>
@@ -882,7 +971,7 @@
         <v>24</v>
       </c>
       <c r="I3" t="n" s="0">
-        <v>24.0</v>
+        <v>60.0</v>
       </c>
       <c r="J3" t="s" s="0">
         <v>25</v>
@@ -917,7 +1006,7 @@
         <v>30</v>
       </c>
       <c r="I4" t="n" s="0">
-        <v>70.0</v>
+        <v>60.0</v>
       </c>
       <c r="J4" t="s" s="0">
         <v>31</v>
@@ -931,39 +1020,39 @@
         <v>33</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>13</v>
+        <v>35</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="F5" t="s" s="0">
         <v>16</v>
       </c>
       <c r="G5" t="s" s="0">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="H5" t="s" s="0">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="I5" t="n" s="0">
-        <v>70.0</v>
+        <v>82.0</v>
       </c>
       <c r="J5" t="s" s="0">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="K5" t="s" s="0">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B6" t="s" s="0">
         <v>12</v>
@@ -975,30 +1064,30 @@
         <v>14</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F6" t="s" s="0">
         <v>16</v>
       </c>
       <c r="G6" t="s" s="0">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H6" t="s" s="0">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="I6" t="n" s="0">
-        <v>70.0</v>
+        <v>40.0</v>
       </c>
       <c r="J6" t="s" s="0">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="K6" t="s" s="0">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B7" t="s" s="0">
         <v>12</v>
@@ -1010,30 +1099,30 @@
         <v>14</v>
       </c>
       <c r="E7" t="s" s="0">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F7" t="s" s="0">
         <v>16</v>
       </c>
       <c r="G7" t="s" s="0">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="H7" t="s" s="0">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="I7" t="n" s="0">
-        <v>40.0</v>
+        <v>24.0</v>
       </c>
       <c r="J7" t="s" s="0">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="K7" t="s" s="0">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B8" t="s" s="0">
         <v>12</v>
@@ -1045,30 +1134,30 @@
         <v>14</v>
       </c>
       <c r="E8" t="s" s="0">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F8" t="s" s="0">
         <v>16</v>
       </c>
       <c r="G8" t="s" s="0">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="H8" t="s" s="0">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I8" t="n" s="0">
         <v>70.0</v>
       </c>
       <c r="J8" t="s" s="0">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="K8" t="s" s="0">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B9" t="s" s="0">
         <v>12</v>
@@ -1086,24 +1175,24 @@
         <v>16</v>
       </c>
       <c r="G9" t="s" s="0">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="H9" t="s" s="0">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="I9" t="n" s="0">
         <v>70.0</v>
       </c>
       <c r="J9" t="s" s="0">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="K9" t="s" s="0">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B10" t="s" s="0">
         <v>12</v>
@@ -1121,24 +1210,24 @@
         <v>16</v>
       </c>
       <c r="G10" t="s" s="0">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="H10" t="s" s="0">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I10" t="n" s="0">
         <v>70.0</v>
       </c>
       <c r="J10" t="s" s="0">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="K10" t="s" s="0">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B11" t="s" s="0">
         <v>12</v>
@@ -1156,24 +1245,24 @@
         <v>16</v>
       </c>
       <c r="G11" t="s" s="0">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H11" t="s" s="0">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I11" t="n" s="0">
-        <v>20.0</v>
+        <v>40.0</v>
       </c>
       <c r="J11" t="s" s="0">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="K11" t="s" s="0">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B12" t="s" s="0">
         <v>12</v>
@@ -1191,24 +1280,24 @@
         <v>16</v>
       </c>
       <c r="G12" t="s" s="0">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="H12" t="s" s="0">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I12" t="n" s="0">
-        <v>60.0</v>
+        <v>70.0</v>
       </c>
       <c r="J12" t="s" s="0">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K12" t="s" s="0">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B13" t="s" s="0">
         <v>12</v>
@@ -1220,30 +1309,30 @@
         <v>14</v>
       </c>
       <c r="E13" t="s" s="0">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F13" t="s" s="0">
         <v>16</v>
       </c>
       <c r="G13" t="s" s="0">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="H13" t="s" s="0">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="I13" t="n" s="0">
-        <v>30.0</v>
+        <v>70.0</v>
       </c>
       <c r="J13" t="s" s="0">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="K13" t="s" s="0">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B14" t="s" s="0">
         <v>12</v>
@@ -1255,30 +1344,30 @@
         <v>14</v>
       </c>
       <c r="E14" t="s" s="0">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F14" t="s" s="0">
         <v>16</v>
       </c>
       <c r="G14" t="s" s="0">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="H14" t="s" s="0">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I14" t="n" s="0">
-        <v>20.0</v>
+        <v>70.0</v>
       </c>
       <c r="J14" t="s" s="0">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="K14" t="s" s="0">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B15" t="s" s="0">
         <v>12</v>
@@ -1290,30 +1379,30 @@
         <v>14</v>
       </c>
       <c r="E15" t="s" s="0">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F15" t="s" s="0">
         <v>16</v>
       </c>
       <c r="G15" t="s" s="0">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="H15" t="s" s="0">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="I15" t="n" s="0">
         <v>20.0</v>
       </c>
       <c r="J15" t="s" s="0">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="K15" t="s" s="0">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B16" t="s" s="0">
         <v>12</v>
@@ -1325,480 +1414,620 @@
         <v>14</v>
       </c>
       <c r="E16" t="s" s="0">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F16" t="s" s="0">
         <v>16</v>
       </c>
       <c r="G16" t="s" s="0">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="H16" t="s" s="0">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="I16" t="n" s="0">
-        <v>30.0</v>
+        <v>60.0</v>
       </c>
       <c r="J16" t="s" s="0">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="K16" t="s" s="0">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>98</v>
+        <v>12</v>
       </c>
       <c r="C17" t="s" s="0">
-        <v>99</v>
+        <v>13</v>
       </c>
       <c r="D17" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E17" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="F17" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="G17" t="s" s="0">
         <v>100</v>
       </c>
-      <c r="E17" t="s" s="0">
-        <v>62</v>
-      </c>
-      <c r="F17" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="G17" t="s" s="0">
+      <c r="H17" t="s" s="0">
         <v>101</v>
       </c>
-      <c r="H17" t="s" s="0">
+      <c r="I17" t="n" s="0">
+        <v>30.0</v>
+      </c>
+      <c r="J17" t="s" s="0">
         <v>102</v>
       </c>
-      <c r="I17" t="n" s="0">
-        <v>60.0</v>
-      </c>
-      <c r="J17" t="s" s="0">
+      <c r="K17" t="s" s="0">
         <v>103</v>
-      </c>
-      <c r="K17" t="s" s="0">
-        <v>104</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
+        <v>104</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C18" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="D18" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E18" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="F18" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="G18" t="s" s="0">
         <v>105</v>
       </c>
-      <c r="B18" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="C18" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="D18" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="E18" t="s" s="0">
-        <v>67</v>
-      </c>
-      <c r="F18" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="G18" t="s" s="0">
+      <c r="H18" t="s" s="0">
         <v>106</v>
       </c>
-      <c r="H18" t="s" s="0">
+      <c r="I18" t="n" s="0">
+        <v>20.0</v>
+      </c>
+      <c r="J18" t="s" s="0">
         <v>107</v>
       </c>
-      <c r="I18" t="n" s="0">
-        <v>50.0</v>
-      </c>
-      <c r="J18" t="s" s="0">
+      <c r="K18" t="s" s="0">
         <v>108</v>
-      </c>
-      <c r="K18" t="s" s="0">
-        <v>109</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
+        <v>109</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C19" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="D19" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E19" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="F19" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="G19" t="s" s="0">
         <v>110</v>
       </c>
-      <c r="B19" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="C19" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="D19" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="E19" t="s" s="0">
-        <v>72</v>
-      </c>
-      <c r="F19" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="G19" t="s" s="0">
+      <c r="H19" t="s" s="0">
         <v>111</v>
       </c>
-      <c r="H19" t="s" s="0">
+      <c r="I19" t="n" s="0">
+        <v>20.0</v>
+      </c>
+      <c r="J19" t="s" s="0">
         <v>112</v>
       </c>
-      <c r="I19" t="n" s="0">
-        <v>81.0</v>
-      </c>
-      <c r="J19" t="s" s="0">
+      <c r="K19" t="s" s="0">
         <v>113</v>
-      </c>
-      <c r="K19" t="s" s="0">
-        <v>114</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
+        <v>114</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C20" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="D20" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E20" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="F20" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="G20" t="s" s="0">
         <v>115</v>
       </c>
-      <c r="B20" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="C20" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="D20" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="E20" t="s" s="0">
-        <v>77</v>
-      </c>
-      <c r="F20" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="G20" t="s" s="0">
+      <c r="H20" t="s" s="0">
         <v>116</v>
       </c>
-      <c r="H20" t="s" s="0">
+      <c r="I20" t="n" s="0">
+        <v>30.0</v>
+      </c>
+      <c r="J20" t="s" s="0">
         <v>117</v>
       </c>
-      <c r="I20" t="n" s="0">
-        <v>60.0</v>
-      </c>
-      <c r="J20" t="s" s="0">
+      <c r="K20" t="s" s="0">
         <v>118</v>
-      </c>
-      <c r="K20" t="s" s="0">
-        <v>119</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
+        <v>119</v>
+      </c>
+      <c r="B21" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="C21" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="D21" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="E21" t="s" s="0">
+        <v>84</v>
+      </c>
+      <c r="F21" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="G21" t="s" s="0">
         <v>120</v>
       </c>
-      <c r="B21" t="s" s="0">
-        <v>98</v>
-      </c>
-      <c r="C21" t="s" s="0">
-        <v>99</v>
-      </c>
-      <c r="D21" t="s" s="0">
-        <v>100</v>
-      </c>
-      <c r="E21" t="s" s="0">
-        <v>82</v>
-      </c>
-      <c r="F21" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="G21" t="s" s="0">
+      <c r="H21" t="s" s="0">
         <v>121</v>
       </c>
-      <c r="H21" t="s" s="0">
+      <c r="I21" t="n" s="0">
+        <v>60.0</v>
+      </c>
+      <c r="J21" t="s" s="0">
         <v>122</v>
       </c>
-      <c r="I21" t="n" s="0">
-        <v>77.0</v>
-      </c>
-      <c r="J21" t="s" s="0">
+      <c r="K21" t="s" s="0">
         <v>123</v>
-      </c>
-      <c r="K21" t="s" s="0">
-        <v>124</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
+        <v>124</v>
+      </c>
+      <c r="B22" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C22" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="D22" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E22" t="s" s="0">
+        <v>89</v>
+      </c>
+      <c r="F22" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="G22" t="s" s="0">
         <v>125</v>
       </c>
-      <c r="B22" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="C22" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="D22" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="E22" t="s" s="0">
-        <v>87</v>
-      </c>
-      <c r="F22" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="G22" t="s" s="0">
+      <c r="H22" t="s" s="0">
         <v>126</v>
-      </c>
-      <c r="H22" t="s" s="0">
-        <v>127</v>
       </c>
       <c r="I22" t="n" s="0">
         <v>50.0</v>
       </c>
       <c r="J22" t="s" s="0">
+        <v>127</v>
+      </c>
+      <c r="K22" t="s" s="0">
         <v>128</v>
-      </c>
-      <c r="K22" t="s" s="0">
-        <v>129</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
+        <v>129</v>
+      </c>
+      <c r="B23" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C23" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="D23" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E23" t="s" s="0">
+        <v>94</v>
+      </c>
+      <c r="F23" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="G23" t="s" s="0">
         <v>130</v>
       </c>
-      <c r="B23" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="C23" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="D23" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="E23" t="s" s="0">
-        <v>92</v>
-      </c>
-      <c r="F23" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="G23" t="s" s="0">
+      <c r="H23" t="s" s="0">
         <v>131</v>
       </c>
-      <c r="H23" t="s" s="0">
+      <c r="I23" t="n" s="0">
+        <v>81.0</v>
+      </c>
+      <c r="J23" t="s" s="0">
         <v>132</v>
       </c>
-      <c r="I23" t="n" s="0">
-        <v>60.0</v>
-      </c>
-      <c r="J23" t="s" s="0">
+      <c r="K23" t="s" s="0">
         <v>133</v>
-      </c>
-      <c r="K23" t="s" s="0">
-        <v>134</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
+        <v>134</v>
+      </c>
+      <c r="B24" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C24" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="D24" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E24" t="s" s="0">
+        <v>99</v>
+      </c>
+      <c r="F24" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="G24" t="s" s="0">
         <v>135</v>
       </c>
-      <c r="B24" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="C24" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="D24" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="E24" t="s" s="0">
-        <v>97</v>
-      </c>
-      <c r="F24" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="G24" t="s" s="0">
+      <c r="H24" t="s" s="0">
         <v>136</v>
       </c>
-      <c r="H24" t="s" s="0">
+      <c r="I24" t="n" s="0">
+        <v>60.0</v>
+      </c>
+      <c r="J24" t="s" s="0">
         <v>137</v>
       </c>
-      <c r="I24" t="n" s="0">
-        <v>30.0</v>
-      </c>
-      <c r="J24" t="s" s="0">
+      <c r="K24" t="s" s="0">
         <v>138</v>
-      </c>
-      <c r="K24" t="s" s="0">
-        <v>139</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
+        <v>139</v>
+      </c>
+      <c r="B25" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="C25" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="D25" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="E25" t="s" s="0">
+        <v>104</v>
+      </c>
+      <c r="F25" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="G25" t="s" s="0">
         <v>140</v>
       </c>
-      <c r="B25" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="C25" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="D25" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="E25" t="s" s="0">
-        <v>105</v>
-      </c>
-      <c r="F25" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="G25" t="s" s="0">
+      <c r="H25" t="s" s="0">
         <v>141</v>
       </c>
-      <c r="H25" t="s" s="0">
+      <c r="I25" t="n" s="0">
+        <v>77.0</v>
+      </c>
+      <c r="J25" t="s" s="0">
         <v>142</v>
       </c>
-      <c r="I25" t="n" s="0">
-        <v>70.0</v>
-      </c>
-      <c r="J25" t="s" s="0">
+      <c r="K25" t="s" s="0">
         <v>143</v>
-      </c>
-      <c r="K25" t="s" s="0">
-        <v>144</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
+        <v>144</v>
+      </c>
+      <c r="B26" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C26" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="D26" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E26" t="s" s="0">
+        <v>109</v>
+      </c>
+      <c r="F26" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="G26" t="s" s="0">
         <v>145</v>
       </c>
-      <c r="B26" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="C26" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="D26" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="E26" t="s" s="0">
-        <v>110</v>
-      </c>
-      <c r="F26" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="G26" t="s" s="0">
+      <c r="H26" t="s" s="0">
         <v>146</v>
       </c>
-      <c r="H26" t="s" s="0">
+      <c r="I26" t="n" s="0">
+        <v>50.0</v>
+      </c>
+      <c r="J26" t="s" s="0">
         <v>147</v>
       </c>
-      <c r="I26" t="n" s="0">
-        <v>87.0</v>
-      </c>
-      <c r="J26" t="s" s="0">
+      <c r="K26" t="s" s="0">
         <v>148</v>
-      </c>
-      <c r="K26" t="s" s="0">
-        <v>149</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
+        <v>149</v>
+      </c>
+      <c r="B27" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C27" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="D27" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E27" t="s" s="0">
+        <v>114</v>
+      </c>
+      <c r="F27" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="G27" t="s" s="0">
         <v>150</v>
       </c>
-      <c r="B27" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="C27" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="D27" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="E27" t="s" s="0">
-        <v>115</v>
-      </c>
-      <c r="F27" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="G27" t="s" s="0">
+      <c r="H27" t="s" s="0">
         <v>151</v>
       </c>
-      <c r="H27" t="s" s="0">
+      <c r="I27" t="n" s="0">
+        <v>60.0</v>
+      </c>
+      <c r="J27" t="s" s="0">
         <v>152</v>
       </c>
-      <c r="I27" t="n" s="0">
-        <v>6.0</v>
-      </c>
-      <c r="J27" t="s" s="0">
+      <c r="K27" t="s" s="0">
         <v>153</v>
-      </c>
-      <c r="K27" t="s" s="0">
-        <v>154</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
+        <v>154</v>
+      </c>
+      <c r="B28" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C28" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="D28" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E28" t="s" s="0">
+        <v>119</v>
+      </c>
+      <c r="F28" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="G28" t="s" s="0">
         <v>155</v>
       </c>
-      <c r="B28" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="C28" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="D28" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="E28" t="s" s="0">
-        <v>120</v>
-      </c>
-      <c r="F28" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="G28" t="s" s="0">
+      <c r="H28" t="s" s="0">
         <v>156</v>
       </c>
-      <c r="H28" t="s" s="0">
+      <c r="I28" t="n" s="0">
+        <v>30.0</v>
+      </c>
+      <c r="J28" t="s" s="0">
         <v>157</v>
       </c>
-      <c r="I28" t="n" s="0">
-        <v>40.0</v>
-      </c>
-      <c r="J28" t="s" s="0">
+      <c r="K28" t="s" s="0">
         <v>158</v>
-      </c>
-      <c r="K28" t="s" s="0">
-        <v>159</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
+        <v>159</v>
+      </c>
+      <c r="B29" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C29" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="D29" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E29" t="s" s="0">
+        <v>124</v>
+      </c>
+      <c r="F29" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="G29" t="s" s="0">
         <v>160</v>
       </c>
-      <c r="B29" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="C29" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="D29" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="E29" t="s" s="0">
-        <v>125</v>
-      </c>
-      <c r="F29" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="G29" t="s" s="0">
+      <c r="H29" t="s" s="0">
         <v>161</v>
       </c>
-      <c r="H29" t="s" s="0">
+      <c r="I29" t="n" s="0">
+        <v>70.0</v>
+      </c>
+      <c r="J29" t="s" s="0">
         <v>162</v>
       </c>
-      <c r="I29" t="n" s="0">
+      <c r="K29" t="s" s="0">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s" s="0">
+        <v>164</v>
+      </c>
+      <c r="B30" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C30" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="D30" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E30" t="s" s="0">
+        <v>129</v>
+      </c>
+      <c r="F30" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="G30" t="s" s="0">
+        <v>165</v>
+      </c>
+      <c r="H30" t="s" s="0">
+        <v>166</v>
+      </c>
+      <c r="I30" t="n" s="0">
+        <v>87.0</v>
+      </c>
+      <c r="J30" t="s" s="0">
+        <v>167</v>
+      </c>
+      <c r="K30" t="s" s="0">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s" s="0">
+        <v>169</v>
+      </c>
+      <c r="B31" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C31" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="D31" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E31" t="s" s="0">
+        <v>134</v>
+      </c>
+      <c r="F31" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="G31" t="s" s="0">
+        <v>170</v>
+      </c>
+      <c r="H31" t="s" s="0">
+        <v>171</v>
+      </c>
+      <c r="I31" t="n" s="0">
+        <v>6.0</v>
+      </c>
+      <c r="J31" t="s" s="0">
+        <v>172</v>
+      </c>
+      <c r="K31" t="s" s="0">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s" s="0">
+        <v>174</v>
+      </c>
+      <c r="B32" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C32" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="D32" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E32" t="s" s="0">
+        <v>139</v>
+      </c>
+      <c r="F32" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="G32" t="s" s="0">
+        <v>175</v>
+      </c>
+      <c r="H32" t="s" s="0">
+        <v>176</v>
+      </c>
+      <c r="I32" t="n" s="0">
         <v>40.0</v>
       </c>
-      <c r="J29" t="s" s="0">
-        <v>163</v>
-      </c>
-      <c r="K29" t="s" s="0">
-        <v>164</v>
+      <c r="J32" t="s" s="0">
+        <v>177</v>
+      </c>
+      <c r="K32" t="s" s="0">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s" s="0">
+        <v>179</v>
+      </c>
+      <c r="B33" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C33" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="D33" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E33" t="s" s="0">
+        <v>144</v>
+      </c>
+      <c r="F33" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="G33" t="s" s="0">
+        <v>180</v>
+      </c>
+      <c r="H33" t="s" s="0">
+        <v>181</v>
+      </c>
+      <c r="I33" t="n" s="0">
+        <v>40.0</v>
+      </c>
+      <c r="J33" t="s" s="0">
+        <v>182</v>
+      </c>
+      <c r="K33" t="s" s="0">
+        <v>183</v>
       </c>
     </row>
   </sheetData>

</xml_diff>